<commit_message>
Actualización automática de datos DGT (2026-07-10)
</commit_message>
<xml_diff>
--- a/Observatorio_Trafico_Marbella_DGT.xlsx
+++ b/Observatorio_Trafico_Marbella_DGT.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portada" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="General_Marbella" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Siniestralidad_Marbella" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sanciones_Marbella" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparativa_2025" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indicadores" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Portada" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="General_Marbella" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Siniestralidad_Marbella" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Sanciones_Marbella" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Comparativa_2025" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Indicadores" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -555,7 +555,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-07-10T11:14:38+00:00</t>
+          <t>2026-07-10T11:31:45+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Aviso por email al detectar datos nuevos (no en el latido mensual)
collect.py escribe data/datahash.txt (firma sha256 de los datasets, sin
el timestamp). El workflow compara la firma antes/después y solo envía
el correo a proyectos1@ammaconsulting.com cuando cambia de verdad.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Observatorio_Trafico_Marbella_DGT.xlsx
+++ b/Observatorio_Trafico_Marbella_DGT.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Portada" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="General_Marbella" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Siniestralidad_Marbella" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Sanciones_Marbella" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Comparativa_2025" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Indicadores" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portada" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="General_Marbella" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Siniestralidad_Marbella" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sanciones_Marbella" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparativa_2025" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indicadores" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -555,7 +555,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-07-10T11:31:45+00:00</t>
+          <t>2026-07-10T11:39:44+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Añadir aforos de tráfico MA-341 y MA-417 (estaciones de aforo)
Nuevo dataset de intensidad de tráfico (ligeros/pesados/total) de las
estaciones MA-341 y MA-417 desde la hoja de seguimiento propia
(data/aforos.csv, mensual 2015-2024 con huecos). collect.py agrega a
totales anuales y conserva el detalle mensual. Se añade sección de
intensidad (anual + estacionalidad), pestaña en el explorador, hoja en
el Excel y un párrafo en el informe PDF.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Observatorio_Trafico_Marbella_DGT.xlsx
+++ b/Observatorio_Trafico_Marbella_DGT.xlsx
@@ -11,8 +11,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="General_Marbella" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Siniestralidad_Marbella" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sanciones_Marbella" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparativa_2025" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indicadores" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aforos_MA341_MA417" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparativa_2025" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indicadores" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -489,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C14"/>
+  <dimension ref="B2:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -555,7 +556,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-07-10T11:39:44+00:00</t>
+          <t>2026-07-13T07:31:49+00:00</t>
         </is>
       </c>
     </row>
@@ -620,6 +621,18 @@
       <c r="C14" t="inlineStr">
         <is>
           <t>2015–2023 (9 años)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Aforos de tráfico MA-341 / MA-417 (seguimiento propio)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2015–2024 (7 años)</t>
         </is>
       </c>
     </row>
@@ -4878,6 +4891,240 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Aforos MA341 MA417</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Ámbito: Marbella  ·  Fuente: DGT en cifras (Información municipal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Indicador</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>2015</v>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>2016</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>2017</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>2018</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>2021</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H4" s="7" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>MA-341 · Ligeros</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="n">
+        <v>976464</v>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>1036714</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>1092052</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>1106548</v>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>1027831</v>
+      </c>
+      <c r="G5" s="9" t="n">
+        <v>1206710</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>1190250</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>MA-341 · Pesados</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>50351</v>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>62893</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>58545</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>60593</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>60319</v>
+      </c>
+      <c r="G6" s="9" t="n">
+        <v>71170</v>
+      </c>
+      <c r="H6" s="9" t="n">
+        <v>85102</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>MA-341 · Total</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>1031065</v>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>1099606</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>1150604</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>1167148</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>1088156</v>
+      </c>
+      <c r="G7" s="9" t="n">
+        <v>1277882</v>
+      </c>
+      <c r="H7" s="9" t="n">
+        <v>1275349</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>MA-417 · Ligeros</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>784465</v>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>825742</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>820513</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>813406</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>737711</v>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>872414</v>
+      </c>
+      <c r="H8" s="9" t="n">
+        <v>884462</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>MA-417 · Pesados</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="n">
+        <v>41831</v>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>38237</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>41941</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>42974</v>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>41092</v>
+      </c>
+      <c r="G9" s="9" t="n">
+        <v>69453</v>
+      </c>
+      <c r="H9" s="9" t="n">
+        <v>76962</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>MA-417 · Total</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>829751</v>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>863979</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>862460</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>856387</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>778812</v>
+      </c>
+      <c r="G10" s="9" t="n">
+        <v>941866</v>
+      </c>
+      <c r="H10" s="9" t="n">
+        <v>961426</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5174,7 +5421,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Añadir criminalidad de Marbella (Ministerio del Interior)
Nuevo dataset de infracciones penales por tipología parseado de los
balances trimestrales oficiales (PDF) del Ministerio del Interior. Cada
balance de Q4 aporta el año + el anterior consolidado; el pipeline nunca
pierde años ya guardados (data/criminalidad.json) y amplía con descargas
espaciadas. Datos 2023-2025 (2024 consolidado). Se añade sección de
criminalidad, pestaña en el explorador, hoja en el Excel y párrafo en el
informe PDF. Requiere pymupdf.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Observatorio_Trafico_Marbella_DGT.xlsx
+++ b/Observatorio_Trafico_Marbella_DGT.xlsx
@@ -12,8 +12,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Siniestralidad_Marbella" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sanciones_Marbella" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aforos_MA341_MA417" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparativa_2025" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indicadores" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criminalidad" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparativa_2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indicadores" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -490,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C15"/>
+  <dimension ref="B2:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -556,7 +557,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-07-13T07:31:49+00:00</t>
+          <t>2026-07-13T09:21:24+00:00</t>
         </is>
       </c>
     </row>
@@ -633,6 +634,18 @@
       <c r="C15" t="inlineStr">
         <is>
           <t>2015–2024 (7 años)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Criminalidad (Ministerio del Interior)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2023–2025 (3 años)</t>
         </is>
       </c>
     </row>
@@ -5125,6 +5138,360 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Criminalidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Ámbito: Marbella  ·  Fuente: DGT en cifras (Información municipal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Indicador</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Criminalidad convencional (total)</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="n">
+        <v>11844</v>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>11988</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>12098</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Homicidios dolosos y asesinatos consumados</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Homicidios dolosos y asesinatos en grado tentativa</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Delitos graves y menos graves de lesiones y riña tumultuaria</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>123</v>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>139</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Secuestro</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Delitos contra la libertad sexual</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>95</v>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>93</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Agresión sexual con penetración</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="n">
+        <v>32</v>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Resto de delitos contra la libertad sexual</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>63</v>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>71</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Robos con violencia e intimidación</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="n">
+        <v>284</v>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>257</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Robos con fuerza en domicilios, establecimientos y otras instalaciones</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="n">
+        <v>817</v>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>686</v>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Robos con fuerza en domicilios</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="n">
+        <v>629</v>
+      </c>
+      <c r="C15" s="9" t="n">
+        <v>523</v>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Hurtos</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="n">
+        <v>3623</v>
+      </c>
+      <c r="C16" s="9" t="n">
+        <v>3749</v>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>3747</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Sustracciones de vehículos</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="n">
+        <v>355</v>
+      </c>
+      <c r="C17" s="9" t="n">
+        <v>364</v>
+      </c>
+      <c r="D17" s="9" t="n">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Tráfico de drogas</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="n">
+        <v>146</v>
+      </c>
+      <c r="C18" s="9" t="n">
+        <v>150</v>
+      </c>
+      <c r="D18" s="9" t="n">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Resto de criminalidad CONVENCIONAL</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="n">
+        <v>6392</v>
+      </c>
+      <c r="C19" s="9" t="n">
+        <v>6544</v>
+      </c>
+      <c r="D19" s="9" t="n">
+        <v>6807</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Cibercriminalidad (total)</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="n">
+        <v>1794</v>
+      </c>
+      <c r="C20" s="9" t="n">
+        <v>1753</v>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>2051</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Estafas informáticas</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="n">
+        <v>1588</v>
+      </c>
+      <c r="C21" s="9" t="n">
+        <v>1483</v>
+      </c>
+      <c r="D21" s="9" t="n">
+        <v>1713</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Otros ciberdelitos</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="n">
+        <v>206</v>
+      </c>
+      <c r="C22" s="9" t="n">
+        <v>270</v>
+      </c>
+      <c r="D22" s="9" t="n">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>TOTAL criminalidad</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="n">
+        <v>13638</v>
+      </c>
+      <c r="C23" s="9" t="n">
+        <v>13741</v>
+      </c>
+      <c r="D23" s="9" t="n">
+        <v>14149</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5421,7 +5788,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Actualización automática de datos DGT (2026-07-13)
</commit_message>
<xml_diff>
--- a/Observatorio_Trafico_Marbella_DGT.xlsx
+++ b/Observatorio_Trafico_Marbella_DGT.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portada" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="General_Marbella" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Siniestralidad_Marbella" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sanciones_Marbella" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aforos_MA341_MA417" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criminalidad" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparativa_2025" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indicadores" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Portada" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="General_Marbella" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Siniestralidad_Marbella" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Sanciones_Marbella" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Aforos_MA341_MA417" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Criminalidad" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Comparativa_2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Indicadores" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -557,7 +557,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-07-13T09:21:24+00:00</t>
+          <t>2026-07-13T09:29:58+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>